<commit_message>
treat as counts total variable instead of bool
</commit_message>
<xml_diff>
--- a/report/tables/clinician_variable_dictionary.xlsx
+++ b/report/tables/clinician_variable_dictionary.xlsx
@@ -19727,7 +19727,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -19737,37 +19737,37 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J256" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t/>
         </is>
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>99.8</t>
+          <t/>
         </is>
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t>0.0: 99.8%; 1.0: 0.2%</t>
+          <t/>
         </is>
       </c>
       <c r="M256" t="inlineStr">
@@ -20266,7 +20266,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -20276,37 +20276,37 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t/>
         </is>
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>99.8</t>
+          <t/>
         </is>
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>0.0: 99.8%; 1.0: 0.2%</t>
+          <t/>
         </is>
       </c>
       <c r="M263" t="inlineStr">
@@ -20343,7 +20343,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
@@ -20353,37 +20353,37 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t/>
         </is>
       </c>
       <c r="K264" t="inlineStr">
         <is>
-          <t>99.7</t>
+          <t/>
         </is>
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>0.0: 99.7%; 1.0: 0.3%</t>
+          <t/>
         </is>
       </c>
       <c r="M264" t="inlineStr">
@@ -20651,7 +20651,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -20661,37 +20661,37 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t/>
         </is>
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>99.8</t>
+          <t/>
         </is>
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>0.0: 99.8%; 1.0: 0.2%</t>
+          <t/>
         </is>
       </c>
       <c r="M268" t="inlineStr">
@@ -20728,7 +20728,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -20738,37 +20738,37 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J269" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t/>
         </is>
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>99.9</t>
+          <t/>
         </is>
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>0.0: 99.9%; 1.0: 0.1%</t>
+          <t/>
         </is>
       </c>
       <c r="M269" t="inlineStr">
@@ -27581,7 +27581,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -27591,37 +27591,37 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J358" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="K358" t="inlineStr">
         <is>
-          <t>60.1</t>
+          <t/>
         </is>
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>1: 60.1%; 0: 39.9%</t>
+          <t/>
         </is>
       </c>
       <c r="M358" t="inlineStr">
@@ -27966,7 +27966,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -27976,37 +27976,37 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J363" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="K363" t="inlineStr">
         <is>
-          <t>99.1</t>
+          <t/>
         </is>
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>0: 99.1%; 1: 0.9%</t>
+          <t/>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -28043,7 +28043,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -28053,37 +28053,37 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J364" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="K364" t="inlineStr">
         <is>
-          <t>96.9</t>
+          <t/>
         </is>
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>0: 96.9%; 1: 3.1%</t>
+          <t/>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -28120,7 +28120,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -28130,37 +28130,37 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J365" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="K365" t="inlineStr">
         <is>
-          <t>94.0</t>
+          <t/>
         </is>
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>0: 94.0%; 1: 6.0%</t>
+          <t/>
         </is>
       </c>
       <c r="M365" t="inlineStr">
@@ -30584,7 +30584,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -30594,37 +30594,37 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t>94.0</t>
+          <t/>
         </is>
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t>0: 94.0%; 1: 6.0%</t>
+          <t/>
         </is>
       </c>
       <c r="M397" t="inlineStr">
@@ -30723,7 +30723,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>dominant_all_cult_org</t>
+          <t>all_cult_bmr_Enterococcus_binary</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -30738,7 +30738,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E399" t="inlineStr">
@@ -30763,32 +30763,32 @@
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J399" t="inlineStr">
         <is>
-          <t>NEGATIVE</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>99.7</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t>NEGATIVE: 39.2%; Escherichia coli: 25.5%; Klebsiella pneumoniae: 6.5%</t>
+          <t>0: 99.7%; 1: 0.3%</t>
         </is>
       </c>
       <c r="M399" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from all_cult_Enterococcus_count, all_cult_Escherichia_coli_count, all_cult_Klebsiella_pneumoniae_count, all_cult_Pseudomonas_aeruginosa_count, all_cult_Staphylococcus_aureus_count, ... (10 source variables): dominant urgent-culture organism: if any organism has combined count &gt;= 2 choose the max; if exactly one organism has count == 1 choose it; otherwise NEGATIVE.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N399" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O399" t="inlineStr">
@@ -30800,7 +30800,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>all_cult_bmr_Enterococcus_binary</t>
+          <t>all_cult_fenotipo_Enterococcus_tuple</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -30815,7 +30815,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
@@ -30840,12 +30840,12 @@
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J400" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
@@ -30855,12 +30855,12 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>0: 99.7%; 1: 0.3%</t>
+          <t>('NEGATIVE',): 99.7%; (9,): 0.2%; (1,): 0.2%</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N400" t="inlineStr">
@@ -30877,7 +30877,7 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo_Enterococcus_tuple</t>
+          <t>all_cult_bmr_Escherichia_coli_binary</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
@@ -30892,7 +30892,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
@@ -30917,27 +30917,27 @@
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J401" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t>99.7</t>
+          <t>87.0</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 99.7%; (9,): 0.2%; (1,): 0.2%</t>
+          <t>0: 87.0%; 1: 13.0%</t>
         </is>
       </c>
       <c r="M401" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N401" t="inlineStr">
@@ -30954,7 +30954,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>all_cult_bmr_Escherichia_coli_binary</t>
+          <t>all_cult_fenotipo_Escherichia_coli_tuple</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
@@ -30969,7 +30969,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E402" t="inlineStr">
@@ -30994,12 +30994,12 @@
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J402" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K402" t="inlineStr">
@@ -31009,12 +31009,12 @@
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t>0: 87.0%; 1: 13.0%</t>
+          <t>('NEGATIVE',): 87.0%; (4,): 2.9%; (9,): 1.6%</t>
         </is>
       </c>
       <c r="M402" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N402" t="inlineStr">
@@ -31031,7 +31031,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo_Escherichia_coli_tuple</t>
+          <t>all_cult_bmr_Klebsiella_pneumoniae_binary</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -31046,7 +31046,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
@@ -31071,27 +31071,27 @@
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J403" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t>87.0</t>
+          <t>96.2</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 87.0%; (4,): 2.9%; (9,): 1.6%</t>
+          <t>0: 96.2%; 1: 3.8%</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N403" t="inlineStr">
@@ -31108,7 +31108,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>all_cult_bmr_Klebsiella_pneumoniae_binary</t>
+          <t>all_cult_fenotipo_Klebsiella_pneumoniae_tuple</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -31123,7 +31123,7 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E404" t="inlineStr">
@@ -31148,12 +31148,12 @@
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>38</t>
         </is>
       </c>
       <c r="J404" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
@@ -31163,12 +31163,12 @@
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>0: 96.2%; 1: 3.8%</t>
+          <t>('NEGATIVE',): 96.2%; (4, 5, 6, 7, 8, 9): 0.7%; (4,): 0.3%</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N404" t="inlineStr">
@@ -31185,7 +31185,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo_Klebsiella_pneumoniae_tuple</t>
+          <t>all_cult_bmr_Pseudomonas_aeruginosa_binary</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -31200,7 +31200,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
@@ -31225,27 +31225,27 @@
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t>96.2</t>
+          <t>99.1</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 96.2%; (4, 5, 6, 7, 8, 9): 0.7%; (4,): 0.3%</t>
+          <t>0: 99.1%; 1: 0.9%</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N405" t="inlineStr">
@@ -31262,7 +31262,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>all_cult_bmr_Pseudomonas_aeruginosa_binary</t>
+          <t>all_cult_fenotipo_Pseudomonas_aeruginosa_tuple</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
@@ -31277,7 +31277,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -31302,12 +31302,12 @@
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J406" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K406" t="inlineStr">
@@ -31317,12 +31317,12 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t>0: 99.1%; 1: 0.9%</t>
+          <t>('NEGATIVE',): 99.1%; (9,): 0.3%; (6,): 0.1%</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N406" t="inlineStr">
@@ -31339,7 +31339,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo_Pseudomonas_aeruginosa_tuple</t>
+          <t>all_cult_bmr_Staphylococcus_aureus_binary</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -31354,7 +31354,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
@@ -31379,27 +31379,27 @@
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t>99.1</t>
+          <t>96.6</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 99.1%; (9,): 0.3%; (6,): 0.1%</t>
+          <t>0: 96.6%; 1: 3.4%</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N407" t="inlineStr">
@@ -31416,7 +31416,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>all_cult_bmr_Staphylococcus_aureus_binary</t>
+          <t>all_cult_fenotipo_Staphylococcus_aureus_tuple</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -31431,7 +31431,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E408" t="inlineStr">
@@ -31456,12 +31456,12 @@
       </c>
       <c r="I408" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J408" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K408" t="inlineStr">
@@ -31471,12 +31471,12 @@
       </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t>0: 96.6%; 1: 3.4%</t>
+          <t>('NEGATIVE',): 96.6%; (1,): 2.0%; (1, 2): 0.7%</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N408" t="inlineStr">
@@ -31493,7 +31493,7 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo_Staphylococcus_aureus_tuple</t>
+          <t>all_cult_bmr_Streptococcus_pneumoniae_binary</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
@@ -31508,7 +31508,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -31533,27 +31533,27 @@
       </c>
       <c r="I409" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J409" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
         <is>
-          <t>96.6</t>
+          <t>99.8</t>
         </is>
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 96.6%; (1,): 2.0%; (1, 2): 0.7%</t>
+          <t>0: 99.8%; 1: 0.2%</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N409" t="inlineStr">
@@ -31570,7 +31570,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>all_cult_bmr_Streptococcus_pneumoniae_binary</t>
+          <t>all_cult_fenotipo_Streptococcus_pneumoniae_tuple</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
@@ -31585,7 +31585,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E410" t="inlineStr">
@@ -31615,7 +31615,7 @@
       </c>
       <c r="J410" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K410" t="inlineStr">
@@ -31625,12 +31625,12 @@
       </c>
       <c r="L410" t="inlineStr">
         <is>
-          <t>0: 99.8%; 1: 0.2%</t>
+          <t>('NEGATIVE',): 99.8%; (1,): 0.2%</t>
         </is>
       </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N410" t="inlineStr">
@@ -31647,7 +31647,7 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo_Streptococcus_pneumoniae_tuple</t>
+          <t>all_cult_bmr__Enterobacteria_binary</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
@@ -31662,7 +31662,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
@@ -31692,22 +31692,22 @@
       </c>
       <c r="J411" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t>99.8</t>
+          <t>96.2</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 99.8%; (1,): 0.2%</t>
+          <t>0: 96.2%; 1: 3.8%</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N411" t="inlineStr">
@@ -31724,7 +31724,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>all_cult_bmr__Enterobacteria_binary</t>
+          <t>all_cult_fenotipo__Enterobacteria_tuple</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -31739,7 +31739,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -31764,12 +31764,12 @@
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>29</t>
         </is>
       </c>
       <c r="J412" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K412" t="inlineStr">
@@ -31779,12 +31779,12 @@
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t>0: 96.2%; 1: 3.8%</t>
+          <t>('NEGATIVE',): 96.2%; (4,): 1.5%; (9,): 0.5%</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N412" t="inlineStr">
@@ -31801,7 +31801,7 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo__Enterobacteria_tuple</t>
+          <t>all_cult_bmr__Fungi_binary</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
@@ -31816,7 +31816,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
@@ -31841,27 +31841,27 @@
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J413" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t>96.2</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 96.2%; (4,): 1.5%; (9,): 0.5%</t>
+          <t>0: 100.0%</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N413" t="inlineStr">
@@ -31878,7 +31878,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>all_cult_bmr__Fungi_binary</t>
+          <t>all_cult_fenotipo__Fungi_tuple</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
@@ -31893,7 +31893,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E414" t="inlineStr">
@@ -31923,7 +31923,7 @@
       </c>
       <c r="J414" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K414" t="inlineStr">
@@ -31933,12 +31933,12 @@
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t>0: 100.0%</t>
+          <t>('NEGATIVE',): 100.0%</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N414" t="inlineStr">
@@ -31955,7 +31955,7 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo__Fungi_tuple</t>
+          <t>all_cult_bmr__Other_bacteria_binary</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
@@ -31970,7 +31970,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E415" t="inlineStr">
@@ -31995,27 +31995,27 @@
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J415" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K415" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>98.6</t>
         </is>
       </c>
       <c r="L415" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 100.0%</t>
+          <t>0: 98.6%; 1: 1.4%</t>
         </is>
       </c>
       <c r="M415" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N415" t="inlineStr">
@@ -32032,7 +32032,7 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>all_cult_bmr__Other_bacteria_binary</t>
+          <t>all_cult_fenotipo__Other_bacteria_tuple</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
@@ -32047,7 +32047,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
@@ -32072,12 +32072,12 @@
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J416" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K416" t="inlineStr">
@@ -32087,12 +32087,12 @@
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t>0: 98.6%; 1: 1.4%</t>
+          <t>('NEGATIVE',): 98.6%; (2,): 0.5%; (1,): 0.3%</t>
         </is>
       </c>
       <c r="M416" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N416" t="inlineStr">
@@ -32109,7 +32109,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo__Other_bacteria_tuple</t>
+          <t>all_cult_bmr__Virus_binary</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -32124,7 +32124,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
@@ -32149,27 +32149,27 @@
       </c>
       <c r="I417" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J417" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K417" t="inlineStr">
         <is>
-          <t>98.6</t>
+          <t>100.0</t>
         </is>
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 98.6%; (2,): 0.5%; (1,): 0.3%</t>
+          <t>0: 100.0%</t>
         </is>
       </c>
       <c r="M417" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N417" t="inlineStr">
@@ -32186,7 +32186,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>all_cult_bmr__Virus_binary</t>
+          <t>all_cult_fenotipo__Virus_tuple</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -32201,7 +32201,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
@@ -32231,7 +32231,7 @@
       </c>
       <c r="J418" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K418" t="inlineStr">
@@ -32241,12 +32241,12 @@
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t>0: 100.0%</t>
+          <t>('NEGATIVE',): 100.0%</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_bmr_*_binary, otros_cult_bmr_*_binary: combine hemoculture and other-culture organism-specific BMR flags into urgent-culture organism-specific BMR flags. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
         </is>
       </c>
       <c r="N418" t="inlineStr">
@@ -32263,7 +32263,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>all_cult_fenotipo__Virus_tuple</t>
+          <t>recurrencia_precoz</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -32278,7 +32278,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
@@ -32303,32 +32303,32 @@
       </c>
       <c r="I419" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J419" t="inlineStr">
-        <is>
-          <t>('NEGATIVE',)</t>
-        </is>
-      </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>78.2</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 100.0%</t>
+          <t>1: 78.2%; 0: 21.8%</t>
         </is>
       </c>
       <c r="M419" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from hemo_fenotipo_*_tuple, otros_cult_fenotipo_*_tuple: combine hemoculture and other-culture organism-specific phenotype tuples into urgent-culture organism-specific phenotype tuples. Removed from the clinician/model-compatible filtered dataset by the final drop list in data/preprocess_columns_to_drop.txt.</t>
+          <t>Created in cross_table_features from cateter_venoso, derivacion_ventriculoper, hemodialisis_permanente, inmunosupresion, leucemia, ... (15 source variables): create synthetic features after table merge, because they combine patient, infection-history, and risk-factor columns.</t>
         </is>
       </c>
       <c r="N419" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="O419" t="inlineStr">
@@ -32340,7 +32340,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>recurrencia_precoz</t>
+          <t>densidad_inf</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -32355,7 +32355,7 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
@@ -32365,37 +32365,37 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t/>
+          <t>2</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J420" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="K420" t="inlineStr">
         <is>
-          <t>78.2</t>
+          <t/>
         </is>
       </c>
       <c r="L420" t="inlineStr">
         <is>
-          <t>1: 78.2%; 0: 21.8%</t>
+          <t/>
         </is>
       </c>
       <c r="M420" t="inlineStr">
@@ -32417,7 +32417,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>densidad_inf</t>
+          <t>residencia_dialisis</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
@@ -32432,7 +32432,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
@@ -32442,37 +32442,37 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G421" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H421" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I421" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J421" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="K421" t="inlineStr">
         <is>
-          <t/>
+          <t>86.4</t>
         </is>
       </c>
       <c r="L421" t="inlineStr">
         <is>
-          <t/>
+          <t>0: 86.4%; 1: 13.6%</t>
         </is>
       </c>
       <c r="M421" t="inlineStr">
@@ -32494,7 +32494,7 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>residencia_dialisis</t>
+          <t>carga_dispositivos</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
@@ -32509,7 +32509,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
@@ -32519,37 +32519,37 @@
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t/>
+          <t>3</t>
         </is>
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J422" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="K422" t="inlineStr">
         <is>
-          <t>86.4</t>
+          <t/>
         </is>
       </c>
       <c r="L422" t="inlineStr">
         <is>
-          <t>0: 86.4%; 1: 13.6%</t>
+          <t/>
         </is>
       </c>
       <c r="M422" t="inlineStr">
@@ -32571,7 +32571,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>carga_dispositivos</t>
+          <t>total_inmunoriesgo_cat</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
@@ -32606,7 +32606,7 @@
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I423" t="inlineStr">
@@ -32648,7 +32648,7 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>total_inmunoriesgo_cat</t>
+          <t>Enterococcus_total</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
@@ -32683,7 +32683,7 @@
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
@@ -32708,7 +32708,7 @@
       </c>
       <c r="M424" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from cateter_venoso, derivacion_ventriculoper, hemodialisis_permanente, inmunosupresion, leucemia, ... (15 source variables): create synthetic features after table merge, because they combine patient, infection-history, and risk-factor columns.</t>
+          <t>Created in cross_table_features from infprev_*_binary, colo_*_binary: create per-organism history total columns from previous-infection and previous-colonization features only; current hemoculture and other urgent-culture organism features are target-side information and are excluded.</t>
         </is>
       </c>
       <c r="N424" t="inlineStr">
@@ -32725,7 +32725,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Enterococcus_total</t>
+          <t>Escherichia_coli_total</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
@@ -32802,7 +32802,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>Escherichia_coli_total</t>
+          <t>Klebsiella_pneumoniae_total</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
@@ -32879,7 +32879,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Klebsiella_pneumoniae_total</t>
+          <t>Pseudomonas_aeruginosa_total</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
@@ -32956,7 +32956,7 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>Pseudomonas_aeruginosa_total</t>
+          <t>Staphylococcus_aureus_total</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
@@ -33033,7 +33033,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>Staphylococcus_aureus_total</t>
+          <t>Streptococcus_pneumoniae_total</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -33068,7 +33068,7 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
@@ -33110,7 +33110,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Streptococcus_pneumoniae_total</t>
+          <t>_Enterobacteria_total</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -33125,7 +33125,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
@@ -33135,37 +33135,37 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
         <is>
-          <t/>
+          <t>0</t>
         </is>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t/>
+          <t>2</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="J430" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t/>
         </is>
       </c>
       <c r="K430" t="inlineStr">
         <is>
-          <t>99.2</t>
+          <t/>
         </is>
       </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t>0.0: 99.2%; 1.0: 0.8%</t>
+          <t/>
         </is>
       </c>
       <c r="M430" t="inlineStr">
@@ -33187,7 +33187,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>_Enterobacteria_total</t>
+          <t>_Fungi_total</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -33264,7 +33264,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>_Fungi_total</t>
+          <t>_Other_bacteria_total</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -33341,7 +33341,7 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>_Other_bacteria_total</t>
+          <t>_Virus_total</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
@@ -33418,7 +33418,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>_Virus_total</t>
+          <t>sample_weight</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -33433,7 +33433,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
@@ -33443,42 +33443,42 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="G434" t="inlineStr">
         <is>
-          <t>0</t>
+          <t/>
         </is>
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="J434" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="K434" t="inlineStr">
         <is>
-          <t/>
+          <t>100.0</t>
         </is>
       </c>
       <c r="L434" t="inlineStr">
         <is>
-          <t/>
+          <t>1: 100.0%</t>
         </is>
       </c>
       <c r="M434" t="inlineStr">
         <is>
-          <t>Created in cross_table_features from infprev_*_binary, colo_*_binary: create per-organism history total columns from previous-infection and previous-colonization features only; current hemoculture and other urgent-culture organism features are target-side information and are excluded.</t>
+          <t>Created in target_building from row: set uniform sample weight to 1.</t>
         </is>
       </c>
       <c r="N434" t="inlineStr">
@@ -33495,17 +33495,17 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>sample_weight</t>
+          <t>sepsis</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>feature</t>
+          <t>target</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t/>
+          <t>2</t>
         </is>
       </c>
       <c r="D435" t="inlineStr">
@@ -33535,27 +33535,27 @@
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J435" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="K435" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>50.8</t>
         </is>
       </c>
       <c r="L435" t="inlineStr">
         <is>
-          <t>1: 100.0%</t>
+          <t>0: 50.8%; 1: 49.2%</t>
         </is>
       </c>
       <c r="M435" t="inlineStr">
         <is>
-          <t>Created in target_building from row: set uniform sample weight to 1.</t>
+          <t>Role in tbl_sepsis from sepsis: retain source binary sepsis label as prediction target.</t>
         </is>
       </c>
       <c r="N435" t="inlineStr">
@@ -33572,7 +33572,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>sepsis</t>
+          <t>bmr_etiologia</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -33587,7 +33587,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
@@ -33617,22 +33617,22 @@
       </c>
       <c r="J436" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>NEGATIVE</t>
         </is>
       </c>
       <c r="K436" t="inlineStr">
         <is>
-          <t>50.8</t>
+          <t>80.6</t>
         </is>
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t>0: 50.8%; 1: 49.2%</t>
+          <t>NEGATIVE: 80.6%; BMR resistente: 19.4%</t>
         </is>
       </c>
       <c r="M436" t="inlineStr">
         <is>
-          <t>Role in tbl_sepsis from sepsis: retain source binary sepsis label as prediction target.</t>
+          <t>Transformed in tbl_hemocultivo_de_urgencias from id_hemocultivo, fecha_hemocultivo, hemo_positivo_si_no, bmr_etiologia, fenotipo_resistencia: deduplicate per patient/admission/organism; use max hemo_positivo_si_no and bmr_etiologia, collect resistance phenotype codes as tuples. Recoded in target_building from bmr_etiologia: 1.0 becomes BMR resistente, all other values become NEGATIVE.</t>
         </is>
       </c>
       <c r="N436" t="inlineStr">
@@ -33649,7 +33649,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>bmr_etiologia</t>
+          <t>fenotipo_resistencia</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -33659,12 +33659,12 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>tuple</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
@@ -33689,12 +33689,12 @@
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J437" t="inlineStr">
         <is>
-          <t>NEGATIVE</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="K437" t="inlineStr">
@@ -33704,12 +33704,12 @@
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t>NEGATIVE: 80.6%; BMR resistente: 19.4%</t>
+          <t>[]: 80.6%; ['Penicilinas']: 9.6%; ['Cefalosporinas 3/4 gen', 'Penicilinas', 'Quinolonas']: 3.0%</t>
         </is>
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t>Transformed in tbl_hemocultivo_de_urgencias from id_hemocultivo, fecha_hemocultivo, hemo_positivo_si_no, bmr_etiologia, fenotipo_resistencia: deduplicate per patient/admission/organism; use max hemo_positivo_si_no and bmr_etiologia, collect resistance phenotype codes as tuples. Recoded in target_building from bmr_etiologia: 1.0 becomes BMR resistente, all other values become NEGATIVE.</t>
+          <t>Transformed in tbl_hemocultivo_de_urgencias from id_hemocultivo, fecha_hemocultivo, hemo_positivo_si_no, bmr_etiologia, fenotipo_resistencia: deduplicate per patient/admission/organism; use max hemo_positivo_si_no and bmr_etiologia, collect resistance phenotype codes as tuples. Recoded in target_building from fenotipo_resistencia: decode phenotype resistance codes to drug names, map drugs to antimicrobial families, deduplicate, and keep an empty list when no mapped phenotype remains.</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
@@ -33726,7 +33726,7 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>fenotipo_resistencia</t>
+          <t>resultado_hemo_multilabel</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
@@ -33736,7 +33736,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
@@ -33766,27 +33766,27 @@
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>39</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>('NEGATIVE',)</t>
         </is>
       </c>
       <c r="K438" t="inlineStr">
         <is>
-          <t>80.6</t>
+          <t>52.8</t>
         </is>
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t>[]: 80.6%; ['Penicilinas']: 9.6%; ['Cefalosporinas 3/4 gen', 'Penicilinas', 'Quinolonas']: 3.0%</t>
+          <t>('NEGATIVE',): 52.8%; ('Escherichia coli',): 20.2%; ('_Other bacteria',): 5.2%</t>
         </is>
       </c>
       <c r="M438" t="inlineStr">
         <is>
-          <t>Transformed in tbl_hemocultivo_de_urgencias from id_hemocultivo, fecha_hemocultivo, hemo_positivo_si_no, bmr_etiologia, fenotipo_resistencia: deduplicate per patient/admission/organism; use max hemo_positivo_si_no and bmr_etiologia, collect resistance phenotype codes as tuples. Recoded in target_building from fenotipo_resistencia: decode phenotype resistance codes to drug names, map drugs to antimicrobial families, deduplicate, and keep an empty list when no mapped phenotype remains.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo_pre_correccion_clinica: pre-clinician-correction tuple of all positive grouped organisms; NEGATIVE tuple if no positive organism exists.</t>
         </is>
       </c>
       <c r="N438" t="inlineStr">
@@ -33803,7 +33803,7 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>resultado_hemo_multilabel</t>
+          <t>resultado_hemo_mo</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
@@ -33813,12 +33813,12 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>101</t>
         </is>
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>tuple</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
@@ -33843,27 +33843,27 @@
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>101</t>
         </is>
       </c>
       <c r="J439" t="inlineStr">
         <is>
-          <t>('NEGATIVE',)</t>
+          <t>NEGATIVE</t>
         </is>
       </c>
       <c r="K439" t="inlineStr">
         <is>
-          <t>52.8</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="L439" t="inlineStr">
         <is>
-          <t>('NEGATIVE',): 52.8%; ('Escherichia coli',): 20.2%; ('_Other bacteria',): 5.2%</t>
+          <t>NEGATIVE: 53.0%; Escherichia coli: 21.7%; Klebsiella pneumoniae: 5.4%</t>
         </is>
       </c>
       <c r="M439" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo_pre_correccion_clinica: pre-clinician-correction tuple of all positive grouped organisms; NEGATIVE tuple if no positive organism exists.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo_original: scalar original microorganism name with clinician-reviewed co-infection resolution applied; NEGATIVE if no positive original microorganism exists.</t>
         </is>
       </c>
       <c r="N439" t="inlineStr">
@@ -33880,7 +33880,7 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>resultado_hemo_mo</t>
+          <t>resultado_hemo</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -33890,7 +33890,7 @@
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
@@ -33920,7 +33920,7 @@
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J440" t="inlineStr">
@@ -33940,7 +33940,7 @@
       </c>
       <c r="M440" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from microorganismo_original: scalar original microorganism name with clinician-reviewed co-infection resolution applied; NEGATIVE if no positive original microorganism exists.</t>
+          <t>Created in tbl_hemocultivo_de_urgencias from hemo_Enterococcus_binary, hemo_Escherichia_coli_binary, hemo_Klebsiella_pneumoniae_binary, hemo_Pseudomonas_aeruginosa_binary, hemo_Staphylococcus_aureus_binary, ... (9 source variables): scalar dominant organism after clinician co-infection correction; NEGATIVE if no positive non-NEGATIVE organism column exists.</t>
         </is>
       </c>
       <c r="N440" t="inlineStr">
@@ -33957,7 +33957,7 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>resultado_hemo</t>
+          <t>dominant_all_cult_org</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
@@ -33967,7 +33967,7 @@
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
@@ -33997,7 +33997,7 @@
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J441" t="inlineStr">
@@ -34007,17 +34007,17 @@
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t>53.0</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L441" t="inlineStr">
         <is>
-          <t>NEGATIVE: 53.0%; Escherichia coli: 21.7%; Klebsiella pneumoniae: 5.4%</t>
+          <t>NEGATIVE: 39.2%; Escherichia coli: 25.5%; Klebsiella pneumoniae: 6.5%</t>
         </is>
       </c>
       <c r="M441" t="inlineStr">
         <is>
-          <t>Created in tbl_hemocultivo_de_urgencias from hemo_Enterococcus_binary, hemo_Escherichia_coli_binary, hemo_Klebsiella_pneumoniae_binary, hemo_Pseudomonas_aeruginosa_binary, hemo_Staphylococcus_aureus_binary, ... (9 source variables): scalar dominant organism after clinician co-infection correction; NEGATIVE if no positive non-NEGATIVE organism column exists.</t>
+          <t>Created in cross_table_features from all_cult_Enterococcus_count, all_cult_Escherichia_coli_count, all_cult_Klebsiella_pneumoniae_count, all_cult_Pseudomonas_aeruginosa_count, all_cult_Staphylococcus_aureus_count, ... (10 source variables): dominant urgent-culture organism: if any organism has combined count &gt;= 2 choose the max; if exactly one organism has count == 1 choose it; otherwise NEGATIVE.</t>
         </is>
       </c>
       <c r="N441" t="inlineStr">

</xml_diff>

<commit_message>
better explanation for number of classes
</commit_message>
<xml_diff>
--- a/report/tables/clinician_variable_dictionary.xlsx
+++ b/report/tables/clinician_variable_dictionary.xlsx
@@ -33659,7 +33659,7 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>6 exploded labels; 15 row-level combinations</t>
         </is>
       </c>
       <c r="D437" t="inlineStr">
@@ -33736,7 +33736,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10 exploded labels; 39 row-level combinations</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
@@ -34198,7 +34198,7 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>13 exploded labels; 75 row-level combinations</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">

</xml_diff>